<commit_message>
feat: integrate root cost and gear SVGs and update pack UI layout
</commit_message>
<xml_diff>
--- a/game/data/startx_data.xlsx
+++ b/game/data/startx_data.xlsx
@@ -8353,8 +8353,8 @@
           <t>p1_university</t>
         </is>
       </c>
-      <c r="J2" t="n">
-        <v>35</v>
+      <c r="J2">
+        <v>60</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: battle box visuals, card pack and asset updates
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/game/data/startx_data.xlsx
+++ b/game/data/startx_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/frankfan/Desktop/Project/StartX/game/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F297BB3D-93AC-D14C-94BD-E62A38926257}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8849EEEF-51AF-2145-8C0C-37C66CCE95F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19780" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19780" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cards" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="240" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="178">
   <si>
     <t>id</t>
   </si>
@@ -30,6 +30,195 @@
     <t>name</t>
   </si>
   <si>
+    <t>type</t>
+  </si>
+  <si>
+    <t>workTags</t>
+  </si>
+  <si>
+    <t>salary</t>
+  </si>
+  <si>
+    <t>capacity</t>
+  </si>
+  <si>
+    <t>value</t>
+  </si>
+  <si>
+    <t>maxUses</t>
+  </si>
+  <si>
+    <t>hp</t>
+  </si>
+  <si>
+    <t>attack</t>
+  </si>
+  <si>
+    <t>workRequired</t>
+  </si>
+  <si>
+    <t>flavor</t>
+  </si>
+  <si>
+    <t>cost</t>
+  </si>
+  <si>
+    <t>founder</t>
+  </si>
+  <si>
+    <t>创始人</t>
+  </si>
+  <si>
+    <t>employee</t>
+  </si>
+  <si>
+    <t>sales,dev,admin,market,data,finance,any</t>
+  </si>
+  <si>
+    <t>不用给钱，啥都能干。梦想是改变世界，合伙人是自己的猫</t>
+  </si>
+  <si>
+    <t>cash</t>
+  </si>
+  <si>
+    <t>现金</t>
+  </si>
+  <si>
+    <t>resource</t>
+  </si>
+  <si>
+    <t>让你又爱又恨的东西</t>
+  </si>
+  <si>
+    <t>p1_neighborhood</t>
+  </si>
+  <si>
+    <t>居住小区</t>
+  </si>
+  <si>
+    <t>resource_node</t>
+  </si>
+  <si>
+    <t>3-5</t>
+  </si>
+  <si>
+    <t>首批客户就是自己的邻居</t>
+  </si>
+  <si>
+    <t>p1_youth</t>
+  </si>
+  <si>
+    <t>小区青年</t>
+  </si>
+  <si>
+    <t>customer</t>
+  </si>
+  <si>
+    <t>不看牌子，便宜好用就行</t>
+  </si>
+  <si>
+    <t>p1_survey</t>
+  </si>
+  <si>
+    <t>市场调研</t>
+  </si>
+  <si>
+    <t>送10个鸡蛋，消费者会在问卷里说实话吗？</t>
+  </si>
+  <si>
+    <t>p1_customer</t>
+  </si>
+  <si>
+    <t>靠谱青年</t>
+  </si>
+  <si>
+    <t>喜欢买性价比高的产品</t>
+  </si>
+  <si>
+    <t>p1_university</t>
+  </si>
+  <si>
+    <t>大学</t>
+  </si>
+  <si>
+    <t>facility</t>
+  </si>
+  <si>
+    <t>真好，又回到校园了</t>
+  </si>
+  <si>
+    <t>p1_intern</t>
+  </si>
+  <si>
+    <t>实习生</t>
+  </si>
+  <si>
+    <t>any</t>
+  </si>
+  <si>
+    <t>懵懂的眼神，管饭就行</t>
+  </si>
+  <si>
+    <t>p1_wholesale</t>
+  </si>
+  <si>
+    <t>批发市场</t>
+  </si>
+  <si>
+    <t>“能再便宜点吗，不能我走了啊！”</t>
+  </si>
+  <si>
+    <t>p1_rawprod</t>
+  </si>
+  <si>
+    <t>裸奔粗糙产品</t>
+  </si>
+  <si>
+    <t>product</t>
+  </si>
+  <si>
+    <t>就这个价格还要啥自行车</t>
+  </si>
+  <si>
+    <t>p1_marketing</t>
+  </si>
+  <si>
+    <t>营销策划</t>
+  </si>
+  <si>
+    <t>“真正好的产品不需要包装。”但我们的不是</t>
+  </si>
+  <si>
+    <t>p1_package</t>
+  </si>
+  <si>
+    <t>带包装粗糙产品</t>
+  </si>
+  <si>
+    <t>带包装的自行车</t>
+  </si>
+  <si>
+    <t>p1_office</t>
+  </si>
+  <si>
+    <t>办公室</t>
+  </si>
+  <si>
+    <t>联合办公里最便宜的非固定工位，咖啡管够</t>
+  </si>
+  <si>
+    <t>rival1</t>
+  </si>
+  <si>
+    <t>银牌销售员</t>
+  </si>
+  <si>
+    <t>rival</t>
+  </si>
+  <si>
+    <t>原来经常尾随你们的人，就是他。</t>
+  </si>
+  <si>
     <t>requiredIdeaId</t>
   </si>
   <si>
@@ -123,214 +312,58 @@
     <t>招募小区青年</t>
   </si>
   <si>
-    <t>any</t>
-  </si>
-  <si>
-    <t>p1_neighborhood</t>
-  </si>
-  <si>
     <t>false</t>
   </si>
   <si>
-    <t>p1_youth</t>
-  </si>
-  <si>
     <t>p1_make_customer</t>
   </si>
   <si>
-    <t>p1_survey</t>
+    <t>转化靠谱青年</t>
   </si>
   <si>
     <t>true</t>
   </si>
   <si>
-    <t>p1_customer</t>
-  </si>
-  <si>
     <t>p1_recruit_intern</t>
   </si>
   <si>
     <t>招募实习生</t>
   </si>
   <si>
-    <t>p1_university</t>
-  </si>
-  <si>
-    <t>p1_intern</t>
-  </si>
-  <si>
     <t>p1_make_rawprod</t>
   </si>
   <si>
     <t>做出粗糙产品</t>
   </si>
   <si>
-    <t>p1_wholesale</t>
-  </si>
-  <si>
-    <t>p1_rawprod</t>
-  </si>
-  <si>
     <t>p1_package_prod</t>
   </si>
   <si>
-    <t>p1_marketing</t>
-  </si>
-  <si>
-    <t>p1_package</t>
+    <t>包装一下产品</t>
   </si>
   <si>
     <t>p1_cash_pkg_cust</t>
   </si>
   <si>
-    <t>cash</t>
+    <t>说得过去的成交</t>
   </si>
   <si>
     <t>p1_cash_pkg_youth</t>
   </si>
   <si>
+    <t>稍微在乎产品的成交</t>
+  </si>
+  <si>
     <t>p1_cash_raw_cust</t>
   </si>
   <si>
+    <t>稍微在乎客户的成交</t>
+  </si>
+  <si>
     <t>p1_cash_raw_youth</t>
   </si>
   <si>
-    <t>type</t>
-  </si>
-  <si>
-    <t>workTags</t>
-  </si>
-  <si>
-    <t>salary</t>
-  </si>
-  <si>
-    <t>capacity</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
-    <t>maxUses</t>
-  </si>
-  <si>
-    <t>hp</t>
-  </si>
-  <si>
-    <t>attack</t>
-  </si>
-  <si>
-    <t>workRequired</t>
-  </si>
-  <si>
-    <t>flavor</t>
-  </si>
-  <si>
-    <t>cost</t>
-  </si>
-  <si>
-    <t>founder</t>
-  </si>
-  <si>
-    <t>创始人</t>
-  </si>
-  <si>
-    <t>employee</t>
-  </si>
-  <si>
-    <t>sales,dev,admin,market,data,finance,any</t>
-  </si>
-  <si>
-    <t>不用给钱，啥都能干。梦想是改变世界，合伙人是自己的猫</t>
-  </si>
-  <si>
-    <t>现金</t>
-  </si>
-  <si>
-    <t>resource</t>
-  </si>
-  <si>
-    <t>让你又爱又恨的东西</t>
-  </si>
-  <si>
-    <t>居住小区</t>
-  </si>
-  <si>
-    <t>resource_node</t>
-  </si>
-  <si>
-    <t>3-5</t>
-  </si>
-  <si>
-    <t>首批客户就是自己的邻居</t>
-  </si>
-  <si>
-    <t>小区青年</t>
-  </si>
-  <si>
-    <t>customer</t>
-  </si>
-  <si>
-    <t>不看牌子，便宜好用就行</t>
-  </si>
-  <si>
-    <t>市场调研</t>
-  </si>
-  <si>
-    <t>送10个鸡蛋，消费者会在问卷里说实话吗？</t>
-  </si>
-  <si>
-    <t>喜欢买性价比高的产品</t>
-  </si>
-  <si>
-    <t>大学</t>
-  </si>
-  <si>
-    <t>facility</t>
-  </si>
-  <si>
-    <t>真好，又回到校园了</t>
-  </si>
-  <si>
-    <t>实习生</t>
-  </si>
-  <si>
-    <t>懵懂的眼神，管饭就行</t>
-  </si>
-  <si>
-    <t>批发市场</t>
-  </si>
-  <si>
-    <t>“能再便宜点吗，不能我走了啊！”</t>
-  </si>
-  <si>
-    <t>裸奔粗糙产品</t>
-  </si>
-  <si>
-    <t>product</t>
-  </si>
-  <si>
-    <t>就这个价格还要啥自行车</t>
-  </si>
-  <si>
-    <t>营销策划</t>
-  </si>
-  <si>
-    <t>“真正好的产品不需要包装。”但我们的不是</t>
-  </si>
-  <si>
-    <t>带包装粗糙产品</t>
-  </si>
-  <si>
-    <t>带包装的自行车</t>
-  </si>
-  <si>
-    <t>p1_office</t>
-  </si>
-  <si>
-    <t>办公室</t>
-  </si>
-  <si>
-    <t>联合办公里最便宜的非固定工位，咖啡管够</t>
+    <t>粗糙的成交</t>
   </si>
   <si>
     <t>stage</t>
@@ -471,12 +504,6 @@
     <t>车库创业</t>
   </si>
   <si>
-    <t>hiring_fair</t>
-  </si>
-  <si>
-    <t>员工招聘</t>
-  </si>
-  <si>
     <t>channel_pack</t>
   </si>
   <si>
@@ -525,31 +552,11 @@
     <t>战！巨头竞争！</t>
   </si>
   <si>
-    <t>粗糙的成交</t>
+    <t>起步发展</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>稍微在乎客户的成交</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>稍微在乎产品的成交</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>说得过去的成交</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>包装一下产品</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>转化靠谱青年</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>靠谱青年</t>
+    <t>Developemnt_pack</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -897,7 +904,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:M14"/>
+  <dimension ref="A1:M15"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
@@ -912,51 +919,51 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>57</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>58</v>
+        <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>59</v>
+        <v>4</v>
       </c>
       <c r="F1" t="s">
-        <v>60</v>
+        <v>5</v>
       </c>
       <c r="G1" t="s">
-        <v>61</v>
+        <v>6</v>
       </c>
       <c r="H1" t="s">
-        <v>62</v>
+        <v>7</v>
       </c>
       <c r="I1" t="s">
-        <v>63</v>
+        <v>8</v>
       </c>
       <c r="J1" t="s">
-        <v>64</v>
+        <v>9</v>
       </c>
       <c r="K1" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="L1" t="s">
-        <v>66</v>
+        <v>11</v>
       </c>
       <c r="M1" t="s">
-        <v>67</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>70</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>71</v>
+        <v>16</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -968,18 +975,18 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>74</v>
+        <v>20</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -991,35 +998,35 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>75</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>76</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
       <c r="H4" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="L4" t="s">
-        <v>79</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>80</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -1028,35 +1035,35 @@
         <v>10</v>
       </c>
       <c r="L5" t="s">
-        <v>82</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="B6" t="s">
-        <v>83</v>
+        <v>32</v>
       </c>
       <c r="C6" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
       <c r="H6" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="L6" t="s">
-        <v>84</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>173</v>
+        <v>35</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>29</v>
       </c>
       <c r="G7">
         <v>2</v>
@@ -1065,61 +1072,61 @@
         <v>15</v>
       </c>
       <c r="L7" t="s">
-        <v>85</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="B8" t="s">
-        <v>86</v>
+        <v>38</v>
       </c>
       <c r="C8" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="L8" t="s">
-        <v>88</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" t="s">
+        <v>41</v>
+      </c>
+      <c r="B9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="L9" t="s">
         <v>44</v>
-      </c>
-      <c r="B9" t="s">
-        <v>89</v>
-      </c>
-      <c r="C9" t="s">
-        <v>70</v>
-      </c>
-      <c r="D9" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9">
-        <v>1</v>
-      </c>
-      <c r="L9" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" t="s">
+        <v>46</v>
+      </c>
+      <c r="C10" t="s">
+        <v>24</v>
+      </c>
+      <c r="H10" t="s">
+        <v>25</v>
+      </c>
+      <c r="L10" t="s">
         <v>47</v>
-      </c>
-      <c r="B10" t="s">
-        <v>91</v>
-      </c>
-      <c r="C10" t="s">
-        <v>77</v>
-      </c>
-      <c r="H10" t="s">
-        <v>78</v>
-      </c>
-      <c r="L10" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1127,10 +1134,10 @@
         <v>48</v>
       </c>
       <c r="B11" t="s">
-        <v>93</v>
+        <v>49</v>
       </c>
       <c r="C11" t="s">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="G11">
         <v>1</v>
@@ -1139,7 +1146,7 @@
         <v>15</v>
       </c>
       <c r="L11" t="s">
-        <v>95</v>
+        <v>51</v>
       </c>
       <c r="M11">
         <v>1</v>
@@ -1147,30 +1154,30 @@
     </row>
     <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B12" t="s">
-        <v>96</v>
+        <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>77</v>
+        <v>24</v>
       </c>
       <c r="H12" t="s">
-        <v>78</v>
+        <v>25</v>
       </c>
       <c r="L12" t="s">
-        <v>97</v>
+        <v>54</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B13" t="s">
-        <v>98</v>
+        <v>56</v>
       </c>
       <c r="C13" t="s">
-        <v>94</v>
+        <v>50</v>
       </c>
       <c r="G13">
         <v>2</v>
@@ -1179,7 +1186,7 @@
         <v>30</v>
       </c>
       <c r="L13" t="s">
-        <v>99</v>
+        <v>57</v>
       </c>
       <c r="M13">
         <v>2</v>
@@ -1187,19 +1194,45 @@
     </row>
     <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="B14" t="s">
-        <v>101</v>
+        <v>59</v>
       </c>
       <c r="C14" t="s">
-        <v>87</v>
+        <v>39</v>
       </c>
       <c r="E14">
         <v>2</v>
       </c>
       <c r="L14" t="s">
-        <v>102</v>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="15" spans="1:13">
+      <c r="A15" t="s">
+        <v>61</v>
+      </c>
+      <c r="B15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C15" t="s">
+        <v>63</v>
+      </c>
+      <c r="E15">
+        <v>0</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15">
+        <v>0</v>
+      </c>
+      <c r="I15">
+        <v>2</v>
+      </c>
+      <c r="L15" t="s">
+        <v>64</v>
       </c>
     </row>
   </sheetData>
@@ -1225,117 +1258,117 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>65</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>66</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>67</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>68</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>69</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>70</v>
       </c>
       <c r="I1" t="s">
-        <v>8</v>
+        <v>71</v>
       </c>
       <c r="J1" t="s">
-        <v>9</v>
+        <v>72</v>
       </c>
       <c r="K1" t="s">
-        <v>10</v>
+        <v>73</v>
       </c>
       <c r="L1" t="s">
-        <v>11</v>
+        <v>74</v>
       </c>
       <c r="M1" t="s">
-        <v>12</v>
+        <v>75</v>
       </c>
       <c r="N1" t="s">
-        <v>13</v>
+        <v>76</v>
       </c>
       <c r="O1" t="s">
-        <v>14</v>
+        <v>77</v>
       </c>
       <c r="P1" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="Q1" t="s">
-        <v>16</v>
+        <v>79</v>
       </c>
       <c r="R1" t="s">
-        <v>17</v>
+        <v>80</v>
       </c>
       <c r="S1" t="s">
-        <v>18</v>
+        <v>81</v>
       </c>
       <c r="T1" t="s">
-        <v>19</v>
+        <v>82</v>
       </c>
       <c r="U1" t="s">
-        <v>20</v>
+        <v>83</v>
       </c>
       <c r="V1" t="s">
-        <v>21</v>
+        <v>84</v>
       </c>
       <c r="W1" t="s">
-        <v>22</v>
+        <v>85</v>
       </c>
       <c r="X1" t="s">
-        <v>23</v>
+        <v>86</v>
       </c>
       <c r="Y1" t="s">
-        <v>24</v>
+        <v>87</v>
       </c>
       <c r="Z1" t="s">
-        <v>25</v>
+        <v>88</v>
       </c>
       <c r="AA1" t="s">
-        <v>26</v>
+        <v>89</v>
       </c>
       <c r="AB1" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="AC1" t="s">
-        <v>28</v>
+        <v>91</v>
       </c>
       <c r="AD1" t="s">
-        <v>29</v>
+        <v>92</v>
       </c>
       <c r="AE1" t="s">
-        <v>30</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:31">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
-        <v>32</v>
+        <v>95</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="E2">
         <v>10</v>
       </c>
       <c r="F2" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="G2">
         <v>1</v>
       </c>
       <c r="H2" t="s">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="U2" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="V2">
         <v>1</v>
@@ -1343,34 +1376,34 @@
     </row>
     <row r="3" spans="1:31">
       <c r="A3" t="s">
-        <v>37</v>
+        <v>97</v>
       </c>
       <c r="B3" t="s">
-        <v>172</v>
+        <v>98</v>
       </c>
       <c r="E3">
         <v>15</v>
       </c>
       <c r="F3" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="G3">
         <v>1</v>
       </c>
       <c r="H3" t="s">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="I3" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="J3">
         <v>1</v>
       </c>
       <c r="K3" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="U3" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="V3">
         <v>1</v>
@@ -1378,28 +1411,28 @@
     </row>
     <row r="4" spans="1:31">
       <c r="A4" t="s">
-        <v>41</v>
+        <v>100</v>
       </c>
       <c r="B4" t="s">
-        <v>42</v>
+        <v>101</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="E4">
         <v>8</v>
       </c>
       <c r="F4" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="G4">
         <v>1</v>
       </c>
       <c r="H4" t="s">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="U4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="V4">
         <v>1</v>
@@ -1407,25 +1440,25 @@
     </row>
     <row r="5" spans="1:31">
       <c r="A5" t="s">
-        <v>45</v>
+        <v>102</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="E5">
         <v>15</v>
       </c>
       <c r="F5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G5">
         <v>1</v>
       </c>
       <c r="H5" t="s">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="U5" t="s">
         <v>48</v>
@@ -1436,10 +1469,10 @@
     </row>
     <row r="6" spans="1:31">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>104</v>
       </c>
       <c r="B6" t="s">
-        <v>171</v>
+        <v>105</v>
       </c>
       <c r="E6">
         <v>30</v>
@@ -1451,19 +1484,19 @@
         <v>1</v>
       </c>
       <c r="H6" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="I6" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="J6">
         <v>1</v>
       </c>
       <c r="K6" t="s">
-        <v>35</v>
+        <v>96</v>
       </c>
       <c r="U6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="V6">
         <v>1</v>
@@ -1471,34 +1504,34 @@
     </row>
     <row r="7" spans="1:31">
       <c r="A7" t="s">
-        <v>52</v>
+        <v>106</v>
       </c>
       <c r="B7" t="s">
-        <v>170</v>
+        <v>107</v>
       </c>
       <c r="E7">
         <v>3</v>
       </c>
       <c r="F7" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G7">
         <v>1</v>
       </c>
       <c r="H7" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="I7" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="J7">
         <v>1</v>
       </c>
       <c r="K7" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="U7" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="V7">
         <v>6</v>
@@ -1506,34 +1539,34 @@
     </row>
     <row r="8" spans="1:31">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>108</v>
       </c>
       <c r="B8" t="s">
-        <v>169</v>
+        <v>109</v>
       </c>
       <c r="E8">
         <v>3</v>
       </c>
       <c r="F8" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="G8">
         <v>1</v>
       </c>
       <c r="H8" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="I8" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="J8">
         <v>1</v>
       </c>
       <c r="K8" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="U8" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="V8">
         <v>5</v>
@@ -1541,10 +1574,10 @@
     </row>
     <row r="9" spans="1:31">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>110</v>
       </c>
       <c r="B9" t="s">
-        <v>168</v>
+        <v>111</v>
       </c>
       <c r="E9">
         <v>3</v>
@@ -1556,19 +1589,19 @@
         <v>1</v>
       </c>
       <c r="H9" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="I9" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="J9">
         <v>1</v>
       </c>
       <c r="K9" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="U9" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="V9">
         <v>5</v>
@@ -1576,10 +1609,10 @@
     </row>
     <row r="10" spans="1:31">
       <c r="A10" t="s">
-        <v>56</v>
+        <v>112</v>
       </c>
       <c r="B10" t="s">
-        <v>167</v>
+        <v>113</v>
       </c>
       <c r="E10">
         <v>3</v>
@@ -1591,19 +1624,19 @@
         <v>1</v>
       </c>
       <c r="H10" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="I10" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="J10">
         <v>1</v>
       </c>
       <c r="K10" t="s">
-        <v>39</v>
+        <v>99</v>
       </c>
       <c r="U10" t="s">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="V10">
         <v>3</v>
@@ -1632,144 +1665,144 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>103</v>
+        <v>114</v>
       </c>
       <c r="D1" t="s">
-        <v>104</v>
+        <v>115</v>
       </c>
       <c r="E1" t="s">
-        <v>105</v>
+        <v>116</v>
       </c>
       <c r="F1" t="s">
-        <v>106</v>
+        <v>117</v>
       </c>
       <c r="G1" t="s">
-        <v>107</v>
+        <v>118</v>
       </c>
       <c r="H1" t="s">
-        <v>108</v>
+        <v>119</v>
       </c>
       <c r="I1" t="s">
-        <v>109</v>
+        <v>120</v>
       </c>
       <c r="J1" t="s">
-        <v>110</v>
+        <v>121</v>
       </c>
       <c r="K1" t="s">
-        <v>111</v>
+        <v>122</v>
       </c>
       <c r="L1" t="s">
-        <v>112</v>
+        <v>123</v>
       </c>
       <c r="M1" t="s">
-        <v>113</v>
+        <v>124</v>
       </c>
       <c r="N1" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="O1" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="P1" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="Q1" t="s">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="R1" t="s">
-        <v>118</v>
+        <v>129</v>
       </c>
       <c r="S1" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="T1" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="U1" t="s">
-        <v>121</v>
+        <v>132</v>
       </c>
       <c r="V1" t="s">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="W1" t="s">
-        <v>123</v>
+        <v>134</v>
       </c>
       <c r="X1" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="Y1" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="Z1" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="AA1" t="s">
-        <v>127</v>
+        <v>138</v>
       </c>
       <c r="AB1" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="AC1" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="AD1" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="AE1" t="s">
-        <v>131</v>
+        <v>142</v>
       </c>
       <c r="AF1" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="AG1" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="AH1" t="s">
-        <v>134</v>
+        <v>145</v>
       </c>
       <c r="AI1" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="AJ1" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="AK1" t="s">
-        <v>137</v>
+        <v>148</v>
       </c>
       <c r="AL1" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="AM1" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="AN1" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="AO1" t="s">
-        <v>141</v>
+        <v>152</v>
       </c>
       <c r="AP1" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="AQ1" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="AR1" t="s">
-        <v>144</v>
+        <v>155</v>
       </c>
       <c r="AS1" t="s">
-        <v>145</v>
+        <v>156</v>
       </c>
       <c r="AT1" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:46">
       <c r="A2" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="B2" t="s">
-        <v>148</v>
+        <v>159</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -1784,49 +1817,49 @@
         <v>4</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>22</v>
       </c>
       <c r="H2">
         <v>40</v>
       </c>
       <c r="I2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="J2">
         <v>60</v>
       </c>
       <c r="K2" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="L2">
         <v>25</v>
       </c>
       <c r="O2" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="P2">
         <v>40</v>
       </c>
       <c r="Q2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="R2">
         <v>35</v>
       </c>
       <c r="S2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="T2">
         <v>25</v>
       </c>
       <c r="W2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="X2">
         <v>40</v>
       </c>
       <c r="Y2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="Z2">
         <v>35</v>
@@ -1838,19 +1871,19 @@
         <v>25</v>
       </c>
       <c r="AE2" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="AF2">
         <v>34</v>
       </c>
       <c r="AG2" t="s">
-        <v>100</v>
+        <v>58</v>
       </c>
       <c r="AH2">
         <v>33</v>
       </c>
       <c r="AI2" t="s">
-        <v>68</v>
+        <v>13</v>
       </c>
       <c r="AJ2">
         <v>33</v>
@@ -1858,10 +1891,10 @@
     </row>
     <row r="3" spans="1:46">
       <c r="A3" t="s">
-        <v>149</v>
+        <v>177</v>
       </c>
       <c r="B3" t="s">
-        <v>150</v>
+        <v>176</v>
       </c>
       <c r="C3">
         <v>1</v>
@@ -1875,13 +1908,19 @@
       <c r="F3">
         <v>5</v>
       </c>
+      <c r="G3" t="s">
+        <v>61</v>
+      </c>
+      <c r="H3">
+        <v>100</v>
+      </c>
     </row>
     <row r="4" spans="1:46">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="B4" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="C4">
         <v>1</v>
@@ -1898,10 +1937,10 @@
     </row>
     <row r="5" spans="1:46">
       <c r="A5" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="B5" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="C5">
         <v>2</v>
@@ -1918,10 +1957,10 @@
     </row>
     <row r="6" spans="1:46">
       <c r="A6" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="B6" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -1938,10 +1977,10 @@
     </row>
     <row r="7" spans="1:46">
       <c r="A7" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="B7" t="s">
-        <v>158</v>
+        <v>167</v>
       </c>
       <c r="C7">
         <v>3</v>
@@ -1958,10 +1997,10 @@
     </row>
     <row r="8" spans="1:46">
       <c r="A8" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="B8" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="C8">
         <v>4</v>
@@ -1978,10 +2017,10 @@
     </row>
     <row r="9" spans="1:46">
       <c r="A9" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="B9" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="C9">
         <v>5</v>
@@ -1998,10 +2037,10 @@
     </row>
     <row r="10" spans="1:46">
       <c r="A10" t="s">
-        <v>163</v>
+        <v>172</v>
       </c>
       <c r="B10" t="s">
-        <v>164</v>
+        <v>173</v>
       </c>
       <c r="C10">
         <v>5</v>
@@ -2018,10 +2057,10 @@
     </row>
     <row r="11" spans="1:46">
       <c r="A11" t="s">
-        <v>165</v>
+        <v>174</v>
       </c>
       <c r="B11" t="s">
-        <v>166</v>
+        <v>175</v>
       </c>
       <c r="C11">
         <v>6</v>

</xml_diff>

<commit_message>
revert: cash output algorithm and tutorial recipe values
</commit_message>
<xml_diff>
--- a/game/data/startx_data.xlsx
+++ b/game/data/startx_data.xlsx
@@ -1344,7 +1344,7 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -1393,7 +1393,7 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="9">
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="V9" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="10">
@@ -1491,7 +1491,7 @@
         </is>
       </c>
       <c r="V10" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update editable background and asset organization
</commit_message>
<xml_diff>
--- a/game/data/startx_data.xlsx
+++ b/game/data/startx_data.xlsx
@@ -1,17 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19960" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19960" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="cards" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="recipes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="packs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cards" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="recipes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="packs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="tasks" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -42,16 +43,21 @@
       <charset val="134"/>
       <family val="3"/>
       <b val="1"/>
-      <color theme="1"/>
+      <color rgb="FFF7F2E8"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF35383A"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -72,8 +78,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -330,13 +340,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N27"/>
+  <dimension ref="A1:N32"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="25.33203125" customWidth="1" min="1" max="1"/>
     <col width="17.1640625" customWidth="1" min="2" max="2"/>
     <col width="15.33203125" customWidth="1" min="3" max="3"/>
-    <col width="14.1640625" bestFit="1" customWidth="1" min="12" max="12"/>
+    <col width="14.1640625" customWidth="1" min="12" max="12"/>
     <col width="56" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
@@ -531,7 +541,7 @@
         <v>1</v>
       </c>
       <c r="L5" s="1" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="M5" t="inlineStr">
         <is>
@@ -584,7 +594,7 @@
         <v>2</v>
       </c>
       <c r="L7" s="1" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -643,7 +653,7 @@
         <v>1</v>
       </c>
       <c r="L9" s="1" t="n">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -686,7 +696,7 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>裸奔粗糙产品</t>
+          <t>粗糙产品</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -698,7 +708,7 @@
         <v>1</v>
       </c>
       <c r="L11" s="1" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="M11" t="inlineStr">
         <is>
@@ -743,7 +753,7 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>带包装粗糙产品</t>
+          <t>带包装的产品</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -876,11 +886,11 @@
         <v>0</v>
       </c>
       <c r="L17" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="M17" s="1" t="inlineStr">
         <is>
-          <t>一份空白的.Docx文件而已。</t>
+          <t>写字楼的特产。</t>
         </is>
       </c>
       <c r="N17" t="n">
@@ -907,7 +917,7 @@
         <v>0</v>
       </c>
       <c r="L18" s="1" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -994,7 +1004,7 @@
         <v>2</v>
       </c>
       <c r="L21" s="1" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="M21" t="inlineStr">
         <is>
@@ -1022,7 +1032,7 @@
         <v>2</v>
       </c>
       <c r="L22" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="23">
@@ -1045,7 +1055,7 @@
         <v>2</v>
       </c>
       <c r="L23" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="24">
@@ -1169,11 +1179,145 @@
         <v>1</v>
       </c>
       <c r="L27" s="1" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="M27" t="inlineStr">
         <is>
           <t>一张干净的桌子和空荡荡的空间。</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>rival2</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>金牌销售员</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>rival</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" t="n">
+        <v>4</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" t="n">
+        <v>4</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>他的销售话术里，每一句都像已经成交。</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>p3_large_neighborhood</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>大型居住小区</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="L29" t="n">
+        <v>60</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>人更多，需求也更多。</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>p3_wholesale_city</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>小商品批发城</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="L30" t="n">
+        <v>60</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>从纽扣到电风扇，这里什么都能找到。</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>p3_bank</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>银行</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>resource</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>钱在这里会安静一点。</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>p3_account</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>账户</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>tool</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" t="n">
+        <v>50</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>余额不是财富，但至少让人睡得着。</t>
         </is>
       </c>
     </row>
@@ -1188,14 +1332,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF22"/>
+  <dimension ref="A1:AF25"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="33.1640625" customWidth="1" min="1" max="1"/>
     <col width="18.83203125" customWidth="1" min="2" max="2"/>
     <col width="28.83203125" customWidth="1" min="3" max="3"/>
-    <col width="13" bestFit="1" customWidth="1" min="5" max="5"/>
-    <col width="10" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24.1640625" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="15.33203125" customWidth="1" min="8" max="8"/>
     <col width="24.1640625" customWidth="1" min="9" max="9"/>
@@ -1366,7 +1510,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="15" customHeight="1">
+    <row r="2" ht="20" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
           <t>p2_specialist_make_customer</t>
@@ -1422,358 +1566,345 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1">
+    <row r="3" ht="20" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
           <t>p2_specialist_package_product</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>采购包装产品</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>产品专员+批发市场+现金</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>p2_product_specialist</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>p1_wholesale</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>p1_package</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>Developemnt_pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>p1_recruit_youth</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>招募小区青年</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>居住小区</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>p1_neighborhood</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>p1_youth</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>garage_pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>p1_make_customer</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>转化靠谱客户</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>市场调研+小区青年</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>p1_survey</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>p1_youth</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="U5" t="inlineStr">
+        <is>
+          <t>p1_customer</t>
+        </is>
+      </c>
+      <c r="V5" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF5" t="inlineStr">
+        <is>
+          <t>garage_pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>p1_recruit_intern</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>招募实习生</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>大学</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>p1_university</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="U6" t="inlineStr">
+        <is>
+          <t>p1_intern</t>
+        </is>
+      </c>
+      <c r="V6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF6" t="inlineStr">
+        <is>
+          <t>garage_pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>p1_make_rawprod</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>采购粗糙产品</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>批发市场+现金+人</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>p1_wholesale</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>p1_rawprod</t>
+        </is>
+      </c>
+      <c r="V7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>garage_pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>p1_package_prod</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>包装粗糙产品</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>产品专员+批发市场+现金</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>p2_product_specialist</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>p1_wholesale</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="M3" t="n">
-        <v>1</v>
-      </c>
-      <c r="N3" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>裸奔粗糙产品+营销策划</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>p1_rawprod</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>true</t>
         </is>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>p1_marketing</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
         <is>
           <t>p1_package</t>
         </is>
       </c>
-      <c r="V3" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF3" t="inlineStr">
-        <is>
-          <t>Developemnt_pack</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>p1_recruit_youth</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>招募小区青年</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>居住小区</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>any</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>p1_neighborhood</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="U4" t="inlineStr">
-        <is>
-          <t>p1_youth</t>
-        </is>
-      </c>
-      <c r="V4" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF4" t="inlineStr">
+      <c r="V8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF8" t="inlineStr">
         <is>
           <t>garage_pack</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>p1_make_customer</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>转化靠谱客户</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>市场调研+小区青年</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>p1_survey</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>p1_youth</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="U5" t="inlineStr">
-        <is>
-          <t>p1_customer</t>
-        </is>
-      </c>
-      <c r="V5" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF5" t="inlineStr">
-        <is>
-          <t>garage_pack</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="15" customHeight="1">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>p1_recruit_intern</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>招募实习生</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>大学</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>any</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>p1_university</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="U6" t="inlineStr">
-        <is>
-          <t>p1_intern</t>
-        </is>
-      </c>
-      <c r="V6" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF6" t="inlineStr">
-        <is>
-          <t>garage_pack</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="15" customHeight="1">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>p1_make_rawprod</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>做出粗糙产品</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>批发市场+现金</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>any</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>p1_wholesale</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>false</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>1</v>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="U7" t="inlineStr">
-        <is>
-          <t>p1_rawprod</t>
-        </is>
-      </c>
-      <c r="V7" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF7" t="inlineStr">
-        <is>
-          <t>garage_pack</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="15" customHeight="1">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>p1_package_prod</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>包装产品</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>裸奔粗糙产品+营销策划+现金</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>p1_rawprod</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>p1_marketing</t>
-        </is>
-      </c>
-      <c r="J8" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>cash</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>1</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="U8" t="inlineStr">
-        <is>
-          <t>p1_package</t>
-        </is>
-      </c>
-      <c r="V8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF8" t="inlineStr">
-        <is>
-          <t>garage_pack</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="15" customHeight="1">
+    <row r="9" ht="20" customHeight="1">
       <c r="A9" t="inlineStr">
         <is>
           <t>p1_cash_pkg_cust</t>
@@ -1829,7 +1960,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1">
+    <row r="10" ht="20" customHeight="1">
       <c r="A10" t="inlineStr">
         <is>
           <t>p1_cash_pkg_youth</t>
@@ -1885,7 +2016,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1">
+    <row r="11" ht="20" customHeight="1">
       <c r="A11" t="inlineStr">
         <is>
           <t>p1_cash_raw_cust</t>
@@ -1941,7 +2072,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1">
+    <row r="12" ht="20" customHeight="1">
       <c r="A12" t="inlineStr">
         <is>
           <t>p1_cash_raw_youth</t>
@@ -1997,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1">
+    <row r="13" ht="20" customHeight="1">
       <c r="A13" t="inlineStr">
         <is>
           <t>p2_make_document</t>
@@ -2045,7 +2176,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1">
+    <row r="14" ht="20" customHeight="1">
       <c r="A14" t="inlineStr">
         <is>
           <t>p2_train_grad</t>
@@ -2101,7 +2232,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1">
+    <row r="15" ht="20" customHeight="1">
       <c r="A15" t="inlineStr">
         <is>
           <t>p2_make_sales_course</t>
@@ -2157,7 +2288,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1">
+    <row r="16" ht="20" customHeight="1">
       <c r="A16" t="inlineStr">
         <is>
           <t>p2_make_product_course</t>
@@ -2213,7 +2344,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15" customHeight="1">
+    <row r="17" ht="20" customHeight="1">
       <c r="A17" t="inlineStr">
         <is>
           <t>p2_make_legal_admin_course</t>
@@ -2269,7 +2400,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1">
+    <row r="18" ht="20" customHeight="1">
       <c r="A18" t="inlineStr">
         <is>
           <t>p2_train_sales_specialist</t>
@@ -2325,7 +2456,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1">
+    <row r="19" ht="20" customHeight="1">
       <c r="A19" t="inlineStr">
         <is>
           <t>p2_train_product_specialist</t>
@@ -2381,7 +2512,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1">
+    <row r="20" ht="20" customHeight="1">
       <c r="A20" t="inlineStr">
         <is>
           <t>p2_train_admin_specialist</t>
@@ -2437,20 +2568,20 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1">
+    <row r="21" ht="20" customHeight="1">
       <c r="A21" t="inlineStr">
         <is>
           <t>p2_build_orderly_workstation</t>
         </is>
       </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>整理办公工位</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="inlineStr">
-        <is>
-          <t>创始人办公桌+行政管理</t>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>增加办公空间</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>创始人办公桌+行政管理+现金</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -2475,6 +2606,19 @@
         <v>1</v>
       </c>
       <c r="K21" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>cash</t>
+        </is>
+      </c>
+      <c r="M21" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" t="inlineStr">
         <is>
           <t>true</t>
         </is>
@@ -2546,6 +2690,189 @@
       <c r="AF22" t="inlineStr">
         <is>
           <t>Developemnt_pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>p3_build_large_neighborhood</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>建设大型居住小区</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>居住小区*2+人员+市场调研</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>p1_neighborhood</t>
+        </is>
+      </c>
+      <c r="G23" t="n">
+        <v>2</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>p1_survey</t>
+        </is>
+      </c>
+      <c r="J23" t="n">
+        <v>1</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>p3_large_neighborhood</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>channel_pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>p3_build_wholesale_city</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>建设小商品批发城</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>批发市场*2+人员+市场调研</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>p1_wholesale</t>
+        </is>
+      </c>
+      <c r="G24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>p1_survey</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
+        <v>1</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>p3_wholesale_city</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>channel_pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>p3_open_account</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>开设账户</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>员工+银行+合同</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>p3_bank</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>false</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>p2_contract</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>p3_account</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>channel_pack</t>
         </is>
       </c>
     </row>
@@ -2560,7 +2887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT11"/>
+  <dimension ref="A1:BD11"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col width="20.83203125" customWidth="1" min="1" max="1"/>
@@ -2798,6 +3125,56 @@
           <t>slot5Prob4</t>
         </is>
       </c>
+      <c r="AU1" t="inlineStr">
+        <is>
+          <t>slot1Card5</t>
+        </is>
+      </c>
+      <c r="AV1" t="inlineStr">
+        <is>
+          <t>slot1Prob5</t>
+        </is>
+      </c>
+      <c r="AW1" t="inlineStr">
+        <is>
+          <t>slot2Card5</t>
+        </is>
+      </c>
+      <c r="AX1" t="inlineStr">
+        <is>
+          <t>slot2Prob5</t>
+        </is>
+      </c>
+      <c r="AY1" t="inlineStr">
+        <is>
+          <t>slot3Card5</t>
+        </is>
+      </c>
+      <c r="AZ1" t="inlineStr">
+        <is>
+          <t>slot3Prob5</t>
+        </is>
+      </c>
+      <c r="BA1" t="inlineStr">
+        <is>
+          <t>slot4Card5</t>
+        </is>
+      </c>
+      <c r="BB1" t="inlineStr">
+        <is>
+          <t>slot4Prob5</t>
+        </is>
+      </c>
+      <c r="BC1" t="inlineStr">
+        <is>
+          <t>slot5Card5</t>
+        </is>
+      </c>
+      <c r="BD1" t="inlineStr">
+        <is>
+          <t>slot5Prob5</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2940,127 +3317,119 @@
         <v>3</v>
       </c>
       <c r="F3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>p1_neighborhood</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>p1_wholesale</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>30</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>p2_law_firm</t>
+        </is>
+      </c>
+      <c r="L3" t="n">
+        <v>25</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>p1_university</t>
+        </is>
+      </c>
+      <c r="N3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>p2_document</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>p1_intern</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>25</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>p1_survey</t>
+        </is>
+      </c>
+      <c r="T3" t="n">
+        <v>15</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>p1_marketing</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>15</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>p2_grad</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>20</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>p2_sales_course</t>
+        </is>
+      </c>
+      <c r="Z3" t="n">
+        <v>20</v>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>p2_product_course</t>
+        </is>
+      </c>
+      <c r="AB3" t="n">
+        <v>20</v>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>p2_legal_admin_course</t>
+        </is>
+      </c>
+      <c r="AD3" t="n">
+        <v>20</v>
+      </c>
+      <c r="AW3" t="inlineStr">
+        <is>
+          <t>p2_admin_management</t>
+        </is>
+      </c>
+      <c r="AX3" t="n">
         <v>5</v>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>p2_law_firm</t>
-        </is>
-      </c>
-      <c r="H3" t="n">
-        <v>55</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>p2_contract</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>45</v>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>p1_intern</t>
-        </is>
-      </c>
-      <c r="P3" t="n">
-        <v>25</v>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>p2_grad</t>
-        </is>
-      </c>
-      <c r="R3" t="n">
+      <c r="AY3" t="inlineStr">
+        <is>
+          <t>p2_document</t>
+        </is>
+      </c>
+      <c r="AZ3" t="n">
         <v>20</v>
-      </c>
-      <c r="S3" t="inlineStr">
-        <is>
-          <t>p2_admin_management</t>
-        </is>
-      </c>
-      <c r="T3" t="n">
-        <v>30</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>p2_orderly_workstation</t>
-        </is>
-      </c>
-      <c r="V3" t="n">
-        <v>25</v>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>p1_survey</t>
-        </is>
-      </c>
-      <c r="X3" t="n">
-        <v>34</v>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>p1_marketing</t>
-        </is>
-      </c>
-      <c r="Z3" t="n">
-        <v>33</v>
-      </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>p2_document</t>
-        </is>
-      </c>
-      <c r="AB3" t="n">
-        <v>33</v>
-      </c>
-      <c r="AE3" t="inlineStr">
-        <is>
-          <t>p2_sales_course</t>
-        </is>
-      </c>
-      <c r="AF3" t="n">
-        <v>34</v>
-      </c>
-      <c r="AG3" t="inlineStr">
-        <is>
-          <t>p2_product_course</t>
-        </is>
-      </c>
-      <c r="AH3" t="n">
-        <v>33</v>
-      </c>
-      <c r="AI3" t="inlineStr">
-        <is>
-          <t>p2_legal_admin_course</t>
-        </is>
-      </c>
-      <c r="AJ3" t="n">
-        <v>33</v>
-      </c>
-      <c r="AM3" t="inlineStr">
-        <is>
-          <t>p2_sales_specialist</t>
-        </is>
-      </c>
-      <c r="AN3" t="n">
-        <v>34</v>
-      </c>
-      <c r="AO3" t="inlineStr">
-        <is>
-          <t>p2_product_specialist</t>
-        </is>
-      </c>
-      <c r="AP3" t="n">
-        <v>33</v>
-      </c>
-      <c r="AQ3" t="inlineStr">
-        <is>
-          <t>p2_admin_specialist</t>
-        </is>
-      </c>
-      <c r="AR3" t="n">
-        <v>33</v>
       </c>
     </row>
     <row r="4">
@@ -3075,7 +3444,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D4" t="n">
         <v>6</v>
@@ -3084,7 +3453,103 @@
         <v>3</v>
       </c>
       <c r="F4" t="n">
-        <v>5</v>
+        <v>3</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>p1_neighborhood</t>
+        </is>
+      </c>
+      <c r="H4" t="n">
+        <v>45</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>p1_wholesale</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>45</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>p2_law_firm</t>
+        </is>
+      </c>
+      <c r="L4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>p3_bank</t>
+        </is>
+      </c>
+      <c r="N4" t="n">
+        <v>10</v>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>p1_survey</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>40</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>p2_grad</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>25</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>p2_sales_specialist</t>
+        </is>
+      </c>
+      <c r="T4" t="n">
+        <v>20</v>
+      </c>
+      <c r="U4" t="inlineStr">
+        <is>
+          <t>p2_product_specialist</t>
+        </is>
+      </c>
+      <c r="V4" t="n">
+        <v>15</v>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>rival2</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>35</v>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>p2_admin_specialist</t>
+        </is>
+      </c>
+      <c r="Z4" t="n">
+        <v>25</v>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>p1_intern</t>
+        </is>
+      </c>
+      <c r="AB4" t="n">
+        <v>25</v>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>p2_document</t>
+        </is>
+      </c>
+      <c r="AD4" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="5">
@@ -3108,7 +3573,7 @@
         <v>3</v>
       </c>
       <c r="F5" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6">
@@ -3132,7 +3597,7 @@
         <v>3</v>
       </c>
       <c r="F6" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="7">
@@ -3156,7 +3621,7 @@
         <v>3</v>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8">
@@ -3180,7 +3645,7 @@
         <v>3</v>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="9">
@@ -3201,10 +3666,10 @@
         <v>24</v>
       </c>
       <c r="E9" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="10">
@@ -3225,10 +3690,10 @@
         <v>34</v>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F10" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11">
@@ -3249,10 +3714,1472 @@
         <v>50</v>
       </c>
       <c r="E11" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J33"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="12.1640625" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="33.33203125" customWidth="1" min="5" max="5"/>
+    <col width="16.6640625" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="7.83203125" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="4" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="B1" s="4" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="C1" s="4" t="inlineStr">
+        <is>
+          <t>group</t>
+        </is>
+      </c>
+      <c r="D1" s="4" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>content</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>triggerType</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>targetId</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>targetCount</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>unlockPack</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>order</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="15" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>main_start</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>主任务</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>创业啦</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>创业啦</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>下定决心这次一定成功</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>game_start</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>main_open_garage</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>主任务</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>创业啦</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>打开车库创业包</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>打开开始卡包</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>pack_opened</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>garage_pack</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Developemnt_pack</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>main_raw_product</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>主任务</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>创业啦</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>初次选货</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>创始人带着一笔现金去批发市场，并生产出粗糙产品</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>founder_recipe</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>p1_make_rawprod</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="2" t="n"/>
+      <c r="J4" s="2" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>main_first_youth</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>主任务</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>创业啦</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>初次找客户</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>将创始人放到居住小区并生产出小区青年</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>founder_recipe</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>p1_recruit_youth</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I5" s="2" t="n"/>
+      <c r="J5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="F11" t="n">
+    </row>
+    <row r="6" ht="15" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>main_first_sale</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>主任务</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>创业啦</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>人生首单</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>将粗糙产品卖给小区青年</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>recipe_complete</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>p1_cash_raw_youth</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>channel_pack</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="n">
         <v>5</v>
+      </c>
+    </row>
+    <row r="7" ht="15" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>main_sell_card</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>主任务</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>创业啦</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>出售一张卡牌</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>将任意可出售卡牌卖出</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>card_sold</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="n"/>
+      <c r="H7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" ht="15" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>main_recruit_intern</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>主任务</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>公司发展</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>你不再孤独了</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>通过大学招募实习生</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>recipe_complete</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>p1_recruit_intern</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>product_pack</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="9" ht="15" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>main_expand_office</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>主任务</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>公司发展</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>办公室扩租</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>空间容量上限首次增加</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>space_increased</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="n"/>
+      <c r="H9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>office_pack</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>main_supply_chain</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>主任务</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>公司发展</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>建立供应链</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>成功连接一条供应链</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>supply_chain_created</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="n"/>
+      <c r="H10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>rival_pack</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" ht="15" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>side_packaged</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>关注客户</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>完成带包装产品</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>生产一张带包装的产品</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>card_produced</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>p1_package</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>side_reliable_customer</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>关注客户</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>找到靠谱客户</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>获得一名靠谱客户</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>card_produced</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>p1_customer</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" s="2" t="n"/>
+      <c r="J12" s="2" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" ht="15" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>side_best_sale</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>关注客户</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>赚更多钱</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>将带包装产品卖给靠谱客户</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>recipe_complete</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>p1_cash_pkg_cust</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>funding_pack</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="14" ht="15" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>org_grad</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>组织发展</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>未来靠你们了</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>将实习生转正为毕业生</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>recipe_complete</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>p2_train_grad</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" ht="30" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>org_sales</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>组织发展</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>销售专员培训完成</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>培养一名销售专员</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>recipe_complete</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>p2_train_sales_specialist</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" ht="30" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>org_product</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>组织发展</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>产品专员培训完成</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>培养一名产品专员</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>recipe_complete</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>p2_train_product_specialist</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" ht="30" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>org_admin</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>组织发展</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>行政专员培训完成</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>培养一名行政专员</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>recipe_complete</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>p2_train_admin_specialist</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>ipo_pack</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" ht="15" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>org_all</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>组织发展</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>组织架构雏形</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>同时拥有销售、产品和行政专员</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>card_state</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>specialists_all</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" ht="30" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>partner_contract</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>合作伙伴</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>让律师事务所出一份合同</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>通过律师事务所起草合同</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>recipe_complete</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>p2_make_contract</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="20" ht="15" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>partner_account</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>合作伙伴</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>让银行开一个账户</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>通过银行开设账户</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>recipe_complete</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>p3_open_account</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="2" t="n"/>
+      <c r="J20" s="2" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21" ht="15" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>battle_one</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>商战</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>友谊为主</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>赶走一名竞争对手</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>rival_defeated</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="n"/>
+      <c r="H21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>international_pack</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="22" ht="30" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>battle_team</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>商战</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>人多力量大</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>多人合力赶走竞争对手</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>team_rival_defeated</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="n"/>
+      <c r="H22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="23" ht="15" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>battle_three</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>商战</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>最好别来</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>累积赶走 3 名竞争对手</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>rival_defeated</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="n"/>
+      <c r="H23" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="24" ht="15" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>battle_ten</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>商战</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>享受竞争</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>累积赶走 10 名竞争对手</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>rival_defeated</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="n"/>
+      <c r="H24" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I24" s="2" t="n"/>
+      <c r="J24" s="2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="25" ht="15" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>battle_twenty</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>商战</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>吵架大师</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>累积赶走 20 名竞争对手</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>rival_defeated</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="n"/>
+      <c r="H25" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>fortune500_pack</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="26" ht="15" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>battle_thirty</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>商战</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>谁敢惹我</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>累积赶走 30 名竞争对手</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>rival_defeated</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="n"/>
+      <c r="H26" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="I26" s="2" t="n"/>
+      <c r="J26" s="2" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>supply_large_home</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>供应链</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>解锁大型居住小区</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>生产大型居住小区</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>card_produced</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>p3_large_neighborhood</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="2" t="n"/>
+      <c r="J27" s="2" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" ht="15" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>supply_wholesale</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>供应链</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>解锁小商品批发城</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>生产小商品批发城</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>card_produced</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>p3_wholesale_city</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I28" s="2" t="n"/>
+      <c r="J28" s="2" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>supply_ten</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>供应链</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>供应链生产 10 次</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>通过供应链累积完成 10 次生产</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>supply_production</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="n"/>
+      <c r="H29" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="I29" s="2" t="n"/>
+      <c r="J29" s="2" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>supply_twenty</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>供应链</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>供应链生产 20 次</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>通过供应链累积完成 20 次生产</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>supply_production</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="n"/>
+      <c r="H30" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="I30" s="2" t="n"/>
+      <c r="J30" s="2" t="n">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="31" ht="15" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>supply_beginner</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>供应链</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>供应链管理新手</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>供应链节点大于等于 3</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>supply_nodes</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="n"/>
+      <c r="H31" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="I31" s="2" t="n"/>
+      <c r="J31" s="2" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="32" ht="15" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>supply_expert</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>供应链</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>供应链管理专家</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="inlineStr">
+        <is>
+          <t>供应链节点大于等于 4</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>supply_nodes</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="n"/>
+      <c r="H32" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="I32" s="2" t="n"/>
+      <c r="J32" s="2" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="33" ht="15" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>supply_master</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>支线任务</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>供应链</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>供应链管理大师</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>供应链节点大于等于 5</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>supply_nodes</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="n"/>
+      <c r="H33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="I33" s="2" t="n"/>
+      <c r="J33" s="2" t="n">
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>